<commit_message>
Update the style in app.py and the data
</commit_message>
<xml_diff>
--- a/data/Vendor_and_Product_details.xlsx
+++ b/data/Vendor_and_Product_details.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="91">
   <si>
     <t>KUNJAL SYNERGIES</t>
   </si>
@@ -98,12 +98,6 @@
     <t>FLORA CHEMICALS</t>
   </si>
   <si>
-    <t>BHARAT JYOTI IMPEX</t>
-  </si>
-  <si>
-    <t>FURNOVA POLYMERS LTD</t>
-  </si>
-  <si>
     <t>IOL CHEMICALS &amp; PHARMACEUTICALS LTD.</t>
   </si>
   <si>
@@ -116,15 +110,9 @@
     <t>NEHA ENTERPRISES</t>
   </si>
   <si>
-    <t>FURFURYL ALCOHOL</t>
-  </si>
-  <si>
     <t>TRIACETIN</t>
   </si>
   <si>
-    <t>LEO CHEMO PLAST</t>
-  </si>
-  <si>
     <t>Product</t>
   </si>
   <si>
@@ -167,9 +155,6 @@
     <t>GUJARAT ALKALIES &amp; CHEMICALS LTD</t>
   </si>
   <si>
-    <t>PTSA</t>
-  </si>
-  <si>
     <t>VANYA INDUSTRIES</t>
   </si>
   <si>
@@ -216,13 +201,109 @@
   </si>
   <si>
     <t xml:space="preserve">CAUSTIC POTASH </t>
+  </si>
+  <si>
+    <t>MAIL_ID</t>
+  </si>
+  <si>
+    <t>monik@sanjaychemindia.com</t>
+  </si>
+  <si>
+    <t>sales@ankitachemical.com</t>
+  </si>
+  <si>
+    <t>info@aprainnovative.in</t>
+  </si>
+  <si>
+    <t>chemicals@mahalaxmigroup.com</t>
+  </si>
+  <si>
+    <t>info@crescentindia.com</t>
+  </si>
+  <si>
+    <t>marketing4@kscl.co.in</t>
+  </si>
+  <si>
+    <t>8693826208/7738068491</t>
+  </si>
+  <si>
+    <t>marketing@lasons.com</t>
+  </si>
+  <si>
+    <t>sales4@prasolchem.com</t>
+  </si>
+  <si>
+    <t>a.s@sahastraa.com</t>
+  </si>
+  <si>
+    <t>info@urmichemicals.in</t>
+  </si>
+  <si>
+    <t>99677 49877</t>
+  </si>
+  <si>
+    <t>97694 48886</t>
+  </si>
+  <si>
+    <t>88502 43739</t>
+  </si>
+  <si>
+    <t>9820071697/9833369934</t>
+  </si>
+  <si>
+    <t>anil@aprainnovative.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PTSA </t>
+  </si>
+  <si>
+    <t>LT 550</t>
+  </si>
+  <si>
+    <t>MOBELCHEM SPECIALTY PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>LT 560</t>
+  </si>
+  <si>
+    <t>ULTIMATE CHEM</t>
+  </si>
+  <si>
+    <t>RUKMINI AGRO SERVICES,SANGLI</t>
+  </si>
+  <si>
+    <t>MS DRUM</t>
+  </si>
+  <si>
+    <t>XETADEL (NEW) TECHNOLOGIES</t>
+  </si>
+  <si>
+    <t>BALMER LAWRIE (NEW)</t>
+  </si>
+  <si>
+    <t>KOLKATA DRUM SUPPLIERS(HENA) OLD</t>
+  </si>
+  <si>
+    <t>IS TRADERS</t>
+  </si>
+  <si>
+    <t>SILICONE TUBE</t>
+  </si>
+  <si>
+    <t>MIDAS SILICONE</t>
+  </si>
+  <si>
+    <t>midas@midasrubber.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -246,20 +327,36 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000001"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,8 +369,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F3F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -311,37 +414,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -355,32 +432,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -663,24 +760,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB94"/>
+  <dimension ref="A1:Z99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" style="7" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="13"/>
-    <col min="4" max="28" width="9.140625" style="1"/>
+    <col min="1" max="1" width="43.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5703125" style="17" customWidth="1"/>
+    <col min="4" max="4" width="37" style="18" customWidth="1"/>
+    <col min="5" max="26" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="4"/>
+    <row r="1" spans="1:26" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -703,138 +805,198 @@
       <c r="X1" s="4"/>
       <c r="Y1" s="4"/>
       <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C2" s="12"/>
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C4" s="12"/>
+      <c r="D4" s="13"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C5" s="12"/>
+      <c r="D5" s="13"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C6" s="14">
+        <v>8369643142</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C7" s="12"/>
+      <c r="D7" s="13"/>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C8" s="16">
+        <v>9821408660</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C9" s="12">
+        <v>9820071697</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="11" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C10" s="12">
+        <v>9819107744</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C11" s="12"/>
+      <c r="D11" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C12" s="12"/>
+      <c r="D12" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C13" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C14" s="12"/>
+      <c r="D14" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="11" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="C15" s="12">
+        <v>9819349444</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="11" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="C16" s="12"/>
+      <c r="D16" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="2"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="13"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -856,18 +1018,16 @@
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
-      <c r="Z18" s="2"/>
-      <c r="AA18" s="2"/>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="2"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -889,18 +1049,16 @@
       <c r="W19" s="2"/>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
-      <c r="Z19" s="2"/>
-      <c r="AA19" s="2"/>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="13"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -922,18 +1080,16 @@
       <c r="W20" s="2"/>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
-      <c r="Z20" s="2"/>
-      <c r="AA20" s="2"/>
-    </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="2"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -955,18 +1111,16 @@
       <c r="W21" s="2"/>
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
-      <c r="Z21" s="2"/>
-      <c r="AA21" s="2"/>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="2"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -988,18 +1142,16 @@
       <c r="W22" s="2"/>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
-      <c r="Z22" s="2"/>
-      <c r="AA22" s="2"/>
-    </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="2"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="13"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1021,18 +1173,16 @@
       <c r="W23" s="2"/>
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
-      <c r="Z23" s="2"/>
-      <c r="AA23" s="2"/>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="2"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="13"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1054,18 +1204,8 @@
       <c r="W24" s="2"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
-      <c r="Z24" s="2"/>
-      <c r="AA24" s="2"/>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="2"/>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1087,18 +1227,16 @@
       <c r="W25" s="2"/>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
-      <c r="Z25" s="2"/>
-      <c r="AA25" s="2"/>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="2"/>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="D26" s="13"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1120,18 +1258,26 @@
       <c r="W26" s="2"/>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
-      <c r="Z26" s="2"/>
-      <c r="AA26" s="2"/>
-    </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="2"/>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="12"/>
+      <c r="D27" s="13"/>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="12"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1153,18 +1299,16 @@
       <c r="W28" s="2"/>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
-      <c r="Z28" s="2"/>
-      <c r="AA28" s="2"/>
-    </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="2"/>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="12"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -1186,18 +1330,16 @@
       <c r="W29" s="2"/>
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
-      <c r="Z29" s="2"/>
-      <c r="AA29" s="2"/>
-    </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="2"/>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="12"/>
+      <c r="D30" s="13"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1219,18 +1361,16 @@
       <c r="W30" s="2"/>
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
-      <c r="Z30" s="2"/>
-      <c r="AA30" s="2"/>
-    </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="14"/>
-      <c r="D31" s="2"/>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="12"/>
+      <c r="D31" s="13"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1252,18 +1392,8 @@
       <c r="W31" s="2"/>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
-      <c r="Z31" s="2"/>
-      <c r="AA31" s="2"/>
-    </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C32" s="14"/>
-      <c r="D32" s="2"/>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1285,18 +1415,30 @@
       <c r="W32" s="2"/>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
-      <c r="Z32" s="2"/>
-      <c r="AA32" s="2"/>
-    </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A33" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B33" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="2"/>
+      <c r="C33" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A34" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="D34" s="13"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1318,18 +1460,18 @@
       <c r="W34" s="2"/>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
-      <c r="Z34" s="2"/>
-      <c r="AA34" s="2"/>
-    </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="2"/>
+      <c r="B35" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="13"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
@@ -1351,18 +1493,8 @@
       <c r="W35" s="2"/>
       <c r="X35" s="2"/>
       <c r="Y35" s="2"/>
-      <c r="Z35" s="2"/>
-      <c r="AA35" s="2"/>
-    </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="2"/>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -1384,18 +1516,18 @@
       <c r="W36" s="2"/>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
-      <c r="Z36" s="2"/>
-      <c r="AA36" s="2"/>
-    </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="2"/>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A37" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="13"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -1417,18 +1549,20 @@
       <c r="W37" s="2"/>
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
-      <c r="Z37" s="2"/>
-      <c r="AA37" s="2"/>
-    </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C38" s="14"/>
-      <c r="D38" s="2"/>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A38" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>75</v>
+      </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -1450,18 +1584,8 @@
       <c r="W38" s="2"/>
       <c r="X38" s="2"/>
       <c r="Y38" s="2"/>
-      <c r="Z38" s="2"/>
-      <c r="AA38" s="2"/>
-    </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="2"/>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -1483,19 +1607,26 @@
       <c r="W39" s="2"/>
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
-      <c r="Z39" s="2"/>
-      <c r="AA39" s="2"/>
-    </row>
-    <row r="40" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C41" s="15"/>
-      <c r="D41" s="5"/>
+    </row>
+    <row r="40" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="12"/>
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="12"/>
+      <c r="D41" s="13"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
@@ -1517,18 +1648,16 @@
       <c r="W41" s="5"/>
       <c r="X41" s="5"/>
       <c r="Y41" s="5"/>
-      <c r="Z41" s="5"/>
-      <c r="AA41" s="5"/>
-    </row>
-    <row r="42" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C42" s="15"/>
-      <c r="D42" s="5"/>
+    </row>
+    <row r="42" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="12"/>
+      <c r="D42" s="13"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
@@ -1550,18 +1679,16 @@
       <c r="W42" s="5"/>
       <c r="X42" s="5"/>
       <c r="Y42" s="5"/>
-      <c r="Z42" s="5"/>
-      <c r="AA42" s="5"/>
-    </row>
-    <row r="43" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="16" t="s">
+    </row>
+    <row r="43" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B43" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C43" s="15"/>
-      <c r="D43" s="5"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="13"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
@@ -1583,19 +1710,17 @@
       <c r="W43" s="5"/>
       <c r="X43" s="5"/>
       <c r="Y43" s="5"/>
-      <c r="Z43" s="5"/>
-      <c r="AA43" s="5"/>
-    </row>
-    <row r="44" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="16" t="s">
+    </row>
+    <row r="44" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B45" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C45" s="15"/>
-      <c r="D45" s="5"/>
+      <c r="B45" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C45" s="12"/>
+      <c r="D45" s="13"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
@@ -1617,18 +1742,16 @@
       <c r="W45" s="5"/>
       <c r="X45" s="5"/>
       <c r="Y45" s="5"/>
-      <c r="Z45" s="5"/>
-      <c r="AA45" s="5"/>
-    </row>
-    <row r="46" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="16" t="s">
+    </row>
+    <row r="46" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B46" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46" s="15"/>
-      <c r="D46" s="5"/>
+      <c r="B46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" s="12"/>
+      <c r="D46" s="13"/>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
@@ -1650,19 +1773,26 @@
       <c r="W46" s="5"/>
       <c r="X46" s="5"/>
       <c r="Y46" s="5"/>
-      <c r="Z46" s="5"/>
-      <c r="AA46" s="5"/>
-    </row>
-    <row r="47" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B48" s="10" t="s">
+    </row>
+    <row r="47" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C48" s="15"/>
-      <c r="D48" s="5"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="13"/>
+    </row>
+    <row r="48" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="12"/>
+      <c r="D48" s="13"/>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
@@ -1684,18 +1814,16 @@
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
       <c r="Y48" s="5"/>
-      <c r="Z48" s="5"/>
-      <c r="AA48" s="5"/>
-    </row>
-    <row r="49" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" s="15"/>
-      <c r="D49" s="5"/>
+    </row>
+    <row r="49" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" s="12"/>
+      <c r="D49" s="13"/>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
@@ -1717,18 +1845,8 @@
       <c r="W49" s="5"/>
       <c r="X49" s="5"/>
       <c r="Y49" s="5"/>
-      <c r="Z49" s="5"/>
-      <c r="AA49" s="5"/>
-    </row>
-    <row r="50" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C50" s="15"/>
-      <c r="D50" s="5"/>
+    </row>
+    <row r="50" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
@@ -1750,18 +1868,16 @@
       <c r="W50" s="5"/>
       <c r="X50" s="5"/>
       <c r="Y50" s="5"/>
-      <c r="Z50" s="5"/>
-      <c r="AA50" s="5"/>
-    </row>
-    <row r="51" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C51" s="15"/>
-      <c r="D51" s="5"/>
+    </row>
+    <row r="51" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" s="12"/>
+      <c r="D51" s="13"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
@@ -1783,59 +1899,73 @@
       <c r="W51" s="5"/>
       <c r="X51" s="5"/>
       <c r="Y51" s="5"/>
-      <c r="Z51" s="5"/>
-      <c r="AA51" s="5"/>
-    </row>
-    <row r="53" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B53" s="10" t="s">
+    </row>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A52" s="20" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="54" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B55" s="10" t="s">
+      <c r="B52" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B56" s="10" t="s">
+      <c r="C52" s="12"/>
+      <c r="D52" s="13"/>
+    </row>
+    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A53" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="12"/>
+      <c r="D53" s="13"/>
+    </row>
+    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A54" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="12"/>
+      <c r="D54" s="13"/>
+    </row>
+    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A56" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="57" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B57" s="10" t="s">
+      <c r="C56" s="12">
+        <v>8347732279</v>
+      </c>
+      <c r="D56" s="13"/>
+    </row>
+    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A57" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="58" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B59" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C59" s="15"/>
-      <c r="D59" s="5"/>
+      <c r="C57" s="12">
+        <v>9326590970</v>
+      </c>
+      <c r="D57" s="13"/>
+    </row>
+    <row r="58" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C59" s="12">
+        <v>9458234520</v>
+      </c>
+      <c r="D59" s="13"/>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
@@ -1857,18 +1987,8 @@
       <c r="W59" s="5"/>
       <c r="X59" s="5"/>
       <c r="Y59" s="5"/>
-      <c r="Z59" s="5"/>
-      <c r="AA59" s="5"/>
-    </row>
-    <row r="60" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B60" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C60" s="15"/>
-      <c r="D60" s="5"/>
+    </row>
+    <row r="60" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
@@ -1890,18 +2010,18 @@
       <c r="W60" s="5"/>
       <c r="X60" s="5"/>
       <c r="Y60" s="5"/>
-      <c r="Z60" s="5"/>
-      <c r="AA60" s="5"/>
-    </row>
-    <row r="61" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B61" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C61" s="15"/>
-      <c r="D61" s="5"/>
+    </row>
+    <row r="61" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="12">
+        <v>9458234520</v>
+      </c>
+      <c r="D61" s="13"/>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
@@ -1923,18 +2043,8 @@
       <c r="W61" s="5"/>
       <c r="X61" s="5"/>
       <c r="Y61" s="5"/>
-      <c r="Z61" s="5"/>
-      <c r="AA61" s="5"/>
-    </row>
-    <row r="62" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B62" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C62" s="15"/>
-      <c r="D62" s="5"/>
+    </row>
+    <row r="62" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
@@ -1956,19 +2066,26 @@
       <c r="W62" s="5"/>
       <c r="X62" s="5"/>
       <c r="Y62" s="5"/>
-      <c r="Z62" s="5"/>
-      <c r="AA62" s="5"/>
-    </row>
-    <row r="63" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B64" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C64" s="15"/>
-      <c r="D64" s="5"/>
+    </row>
+    <row r="63" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B63" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C63" s="12"/>
+      <c r="D63" s="13"/>
+    </row>
+    <row r="64" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B64" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C64" s="12"/>
+      <c r="D64" s="13"/>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
@@ -1990,18 +2107,16 @@
       <c r="W64" s="5"/>
       <c r="X64" s="5"/>
       <c r="Y64" s="5"/>
-      <c r="Z64" s="5"/>
-      <c r="AA64" s="5"/>
-    </row>
-    <row r="65" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B65" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C65" s="15"/>
-      <c r="D65" s="5"/>
+    </row>
+    <row r="65" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C65" s="12"/>
+      <c r="D65" s="13"/>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
@@ -2023,19 +2138,26 @@
       <c r="W65" s="5"/>
       <c r="X65" s="5"/>
       <c r="Y65" s="5"/>
-      <c r="Z65" s="5"/>
-      <c r="AA65" s="5"/>
-    </row>
-    <row r="66" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="67" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B67" s="18" t="s">
+    </row>
+    <row r="66" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C67" s="15"/>
-      <c r="D67" s="5"/>
+      <c r="B66" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C66" s="12"/>
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C67" s="12"/>
+      <c r="D67" s="13"/>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
@@ -2057,18 +2179,16 @@
       <c r="W67" s="5"/>
       <c r="X67" s="5"/>
       <c r="Y67" s="5"/>
-      <c r="Z67" s="5"/>
-      <c r="AA67" s="5"/>
-    </row>
-    <row r="68" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B68" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C68" s="15"/>
-      <c r="D68" s="5"/>
+    </row>
+    <row r="68" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C68" s="12"/>
+      <c r="D68" s="13"/>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
@@ -2090,18 +2210,8 @@
       <c r="W68" s="5"/>
       <c r="X68" s="5"/>
       <c r="Y68" s="5"/>
-      <c r="Z68" s="5"/>
-      <c r="AA68" s="5"/>
-    </row>
-    <row r="69" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B69" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C69" s="15"/>
-      <c r="D69" s="5"/>
+    </row>
+    <row r="69" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
@@ -2123,18 +2233,16 @@
       <c r="W69" s="5"/>
       <c r="X69" s="5"/>
       <c r="Y69" s="5"/>
-      <c r="Z69" s="5"/>
-      <c r="AA69" s="5"/>
-    </row>
-    <row r="70" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B70" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="C70" s="15"/>
-      <c r="D70" s="5"/>
+    </row>
+    <row r="70" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" s="12"/>
+      <c r="D70" s="13"/>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
       <c r="G70" s="5"/>
@@ -2156,18 +2264,16 @@
       <c r="W70" s="5"/>
       <c r="X70" s="5"/>
       <c r="Y70" s="5"/>
-      <c r="Z70" s="5"/>
-      <c r="AA70" s="5"/>
-    </row>
-    <row r="71" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B71" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C71" s="15"/>
-      <c r="D71" s="5"/>
+    </row>
+    <row r="71" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" s="12"/>
+      <c r="D71" s="13"/>
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
@@ -2189,18 +2295,16 @@
       <c r="W71" s="5"/>
       <c r="X71" s="5"/>
       <c r="Y71" s="5"/>
-      <c r="Z71" s="5"/>
-      <c r="AA71" s="5"/>
-    </row>
-    <row r="72" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B72" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C72" s="15"/>
-      <c r="D72" s="5"/>
+    </row>
+    <row r="72" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C72" s="12"/>
+      <c r="D72" s="13"/>
       <c r="E72" s="5"/>
       <c r="F72" s="5"/>
       <c r="G72" s="5"/>
@@ -2222,19 +2326,26 @@
       <c r="W72" s="5"/>
       <c r="X72" s="5"/>
       <c r="Y72" s="5"/>
-      <c r="Z72" s="5"/>
-      <c r="AA72" s="5"/>
-    </row>
-    <row r="73" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="74" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B74" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C74" s="15"/>
-      <c r="D74" s="5"/>
+    </row>
+    <row r="73" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C73" s="12"/>
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C74" s="12"/>
+      <c r="D74" s="13"/>
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
       <c r="G74" s="5"/>
@@ -2256,18 +2367,16 @@
       <c r="W74" s="5"/>
       <c r="X74" s="5"/>
       <c r="Y74" s="5"/>
-      <c r="Z74" s="5"/>
-      <c r="AA74" s="5"/>
-    </row>
-    <row r="75" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B75" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C75" s="15"/>
-      <c r="D75" s="5"/>
+    </row>
+    <row r="75" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C75" s="12"/>
+      <c r="D75" s="13"/>
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
@@ -2289,18 +2398,16 @@
       <c r="W75" s="5"/>
       <c r="X75" s="5"/>
       <c r="Y75" s="5"/>
-      <c r="Z75" s="5"/>
-      <c r="AA75" s="5"/>
-    </row>
-    <row r="76" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B76" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C76" s="15"/>
-      <c r="D76" s="5"/>
+    </row>
+    <row r="76" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C76" s="12"/>
+      <c r="D76" s="13"/>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
@@ -2322,18 +2429,16 @@
       <c r="W76" s="5"/>
       <c r="X76" s="5"/>
       <c r="Y76" s="5"/>
-      <c r="Z76" s="5"/>
-      <c r="AA76" s="5"/>
-    </row>
-    <row r="77" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B77" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C77" s="15"/>
-      <c r="D77" s="5"/>
+    </row>
+    <row r="77" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C77" s="12"/>
+      <c r="D77" s="13"/>
       <c r="E77" s="5"/>
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
@@ -2355,18 +2460,8 @@
       <c r="W77" s="5"/>
       <c r="X77" s="5"/>
       <c r="Y77" s="5"/>
-      <c r="Z77" s="5"/>
-      <c r="AA77" s="5"/>
-    </row>
-    <row r="78" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B78" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C78" s="15"/>
-      <c r="D78" s="5"/>
+    </row>
+    <row r="78" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E78" s="5"/>
       <c r="F78" s="5"/>
       <c r="G78" s="5"/>
@@ -2388,18 +2483,16 @@
       <c r="W78" s="5"/>
       <c r="X78" s="5"/>
       <c r="Y78" s="5"/>
-      <c r="Z78" s="5"/>
-      <c r="AA78" s="5"/>
-    </row>
-    <row r="79" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B79" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C79" s="15"/>
-      <c r="D79" s="5"/>
+    </row>
+    <row r="79" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" s="12"/>
+      <c r="D79" s="13"/>
       <c r="E79" s="5"/>
       <c r="F79" s="5"/>
       <c r="G79" s="5"/>
@@ -2421,18 +2514,16 @@
       <c r="W79" s="5"/>
       <c r="X79" s="5"/>
       <c r="Y79" s="5"/>
-      <c r="Z79" s="5"/>
-      <c r="AA79" s="5"/>
-    </row>
-    <row r="80" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B80" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C80" s="15"/>
-      <c r="D80" s="5"/>
+    </row>
+    <row r="80" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80" s="12"/>
+      <c r="D80" s="13"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
       <c r="G80" s="5"/>
@@ -2454,19 +2545,26 @@
       <c r="W80" s="5"/>
       <c r="X80" s="5"/>
       <c r="Y80" s="5"/>
-      <c r="Z80" s="5"/>
-      <c r="AA80" s="5"/>
-    </row>
-    <row r="81" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="82" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B82" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C82" s="15"/>
-      <c r="D82" s="5"/>
+    </row>
+    <row r="81" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C81" s="12"/>
+      <c r="D81" s="13"/>
+    </row>
+    <row r="82" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C82" s="12"/>
+      <c r="D82" s="13"/>
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
       <c r="G82" s="5"/>
@@ -2488,18 +2586,16 @@
       <c r="W82" s="5"/>
       <c r="X82" s="5"/>
       <c r="Y82" s="5"/>
-      <c r="Z82" s="5"/>
-      <c r="AA82" s="5"/>
-    </row>
-    <row r="83" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B83" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C83" s="15"/>
-      <c r="D83" s="5"/>
+    </row>
+    <row r="83" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C83" s="12"/>
+      <c r="D83" s="13"/>
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
@@ -2521,18 +2617,16 @@
       <c r="W83" s="5"/>
       <c r="X83" s="5"/>
       <c r="Y83" s="5"/>
-      <c r="Z83" s="5"/>
-      <c r="AA83" s="5"/>
-    </row>
-    <row r="84" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B84" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C84" s="15"/>
-      <c r="D84" s="5"/>
+    </row>
+    <row r="84" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C84" s="12"/>
+      <c r="D84" s="13"/>
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
@@ -2554,18 +2648,16 @@
       <c r="W84" s="5"/>
       <c r="X84" s="5"/>
       <c r="Y84" s="5"/>
-      <c r="Z84" s="5"/>
-      <c r="AA84" s="5"/>
-    </row>
-    <row r="85" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B85" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C85" s="15"/>
-      <c r="D85" s="5"/>
+    </row>
+    <row r="85" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85" s="12"/>
+      <c r="D85" s="13"/>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
       <c r="G85" s="5"/>
@@ -2587,18 +2679,16 @@
       <c r="W85" s="5"/>
       <c r="X85" s="5"/>
       <c r="Y85" s="5"/>
-      <c r="Z85" s="5"/>
-      <c r="AA85" s="5"/>
-    </row>
-    <row r="86" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B86" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C86" s="15"/>
-      <c r="D86" s="5"/>
+    </row>
+    <row r="86" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="12"/>
+      <c r="D86" s="13"/>
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
       <c r="G86" s="5"/>
@@ -2620,18 +2710,16 @@
       <c r="W86" s="5"/>
       <c r="X86" s="5"/>
       <c r="Y86" s="5"/>
-      <c r="Z86" s="5"/>
-      <c r="AA86" s="5"/>
-    </row>
-    <row r="87" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B87" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C87" s="15"/>
-      <c r="D87" s="5"/>
+    </row>
+    <row r="87" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C87" s="12"/>
+      <c r="D87" s="13"/>
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="5"/>
@@ -2653,18 +2741,16 @@
       <c r="W87" s="5"/>
       <c r="X87" s="5"/>
       <c r="Y87" s="5"/>
-      <c r="Z87" s="5"/>
-      <c r="AA87" s="5"/>
-    </row>
-    <row r="88" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B88" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C88" s="15"/>
-      <c r="D88" s="5"/>
+    </row>
+    <row r="88" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" s="12"/>
+      <c r="D88" s="13"/>
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
       <c r="G88" s="5"/>
@@ -2686,18 +2772,8 @@
       <c r="W88" s="5"/>
       <c r="X88" s="5"/>
       <c r="Y88" s="5"/>
-      <c r="Z88" s="5"/>
-      <c r="AA88" s="5"/>
-    </row>
-    <row r="89" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B89" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C89" s="15"/>
-      <c r="D89" s="5"/>
+    </row>
+    <row r="89" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
       <c r="G89" s="5"/>
@@ -2719,18 +2795,16 @@
       <c r="W89" s="5"/>
       <c r="X89" s="5"/>
       <c r="Y89" s="5"/>
-      <c r="Z89" s="5"/>
-      <c r="AA89" s="5"/>
-    </row>
-    <row r="90" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B90" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C90" s="15"/>
-      <c r="D90" s="5"/>
+    </row>
+    <row r="90" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C90" s="12"/>
+      <c r="D90" s="13"/>
       <c r="E90" s="5"/>
       <c r="F90" s="5"/>
       <c r="G90" s="5"/>
@@ -2752,19 +2826,26 @@
       <c r="W90" s="5"/>
       <c r="X90" s="5"/>
       <c r="Y90" s="5"/>
-      <c r="Z90" s="5"/>
-      <c r="AA90" s="5"/>
-    </row>
-    <row r="91" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="92" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B92" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C92" s="15"/>
-      <c r="D92" s="5"/>
+    </row>
+    <row r="91" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C91" s="12"/>
+      <c r="D91" s="13"/>
+    </row>
+    <row r="92" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C92" s="12"/>
+      <c r="D92" s="13"/>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
@@ -2786,18 +2867,8 @@
       <c r="W92" s="5"/>
       <c r="X92" s="5"/>
       <c r="Y92" s="5"/>
-      <c r="Z92" s="5"/>
-      <c r="AA92" s="5"/>
-    </row>
-    <row r="93" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B93" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C93" s="15"/>
-      <c r="D93" s="5"/>
+    </row>
+    <row r="93" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
       <c r="G93" s="5"/>
@@ -2819,18 +2890,16 @@
       <c r="W93" s="5"/>
       <c r="X93" s="5"/>
       <c r="Y93" s="5"/>
-      <c r="Z93" s="5"/>
-      <c r="AA93" s="5"/>
-    </row>
-    <row r="94" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B94" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C94" s="15"/>
-      <c r="D94" s="5"/>
+    </row>
+    <row r="94" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C94" s="12"/>
+      <c r="D94" s="13"/>
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
       <c r="G94" s="5"/>
@@ -2852,8 +2921,50 @@
       <c r="W94" s="5"/>
       <c r="X94" s="5"/>
       <c r="Y94" s="5"/>
-      <c r="Z94" s="5"/>
-      <c r="AA94" s="5"/>
+    </row>
+    <row r="95" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A95" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C95" s="12"/>
+      <c r="D95" s="13"/>
+    </row>
+    <row r="96" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A96" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C96" s="12"/>
+      <c r="D96" s="13"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C97" s="12"/>
+      <c r="D97" s="13"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C99" s="12">
+        <v>9825185098</v>
+      </c>
+      <c r="D99" s="13" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>